<commit_message>
update flowchart.xlsx - add new entry
</commit_message>
<xml_diff>
--- a/1.training_model/supplementary/1. Flowchart ML development.xlsx
+++ b/1.training_model/supplementary/1. Flowchart ML development.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sitisyaziyah\source\repos\DeviceCluster\1.training_model\supplementary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{999A732D-812E-4F4C-BD19-9B58B7EDD54C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{172331D7-7552-4EE9-A798-6093142F629F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A3A45E78-3C42-44AE-93A4-41B09245FE7F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{A3A45E78-3C42-44AE-93A4-41B09245FE7F}"/>
   </bookViews>
   <sheets>
     <sheet name="Flowchart ML" sheetId="1" r:id="rId1"/>
     <sheet name="question" sheetId="5" r:id="rId2"/>
-    <sheet name="Parameter Details" sheetId="3" r:id="rId3"/>
-    <sheet name="Movement dataset" sheetId="2" r:id="rId4"/>
-    <sheet name="suppl" sheetId="4" r:id="rId5"/>
+    <sheet name="Sheet2" sheetId="7" r:id="rId3"/>
+    <sheet name="Parameter Details" sheetId="3" r:id="rId4"/>
+    <sheet name="Movement dataset" sheetId="2" r:id="rId5"/>
+    <sheet name="suppl" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -736,18 +737,6 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -776,6 +765,18 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -9337,40 +9338,40 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:38" x14ac:dyDescent="0.35">
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="N2" s="11" t="s">
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="N2" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="O2" s="11"/>
-      <c r="P2" s="11"/>
-      <c r="Q2" s="11"/>
-      <c r="R2" s="11"/>
-      <c r="V2" s="11" t="s">
+      <c r="O2" s="20"/>
+      <c r="P2" s="20"/>
+      <c r="Q2" s="20"/>
+      <c r="R2" s="20"/>
+      <c r="V2" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="W2" s="11"/>
-      <c r="X2" s="11"/>
-      <c r="Y2" s="11"/>
-      <c r="Z2" s="11"/>
-      <c r="AD2" s="11" t="s">
+      <c r="W2" s="20"/>
+      <c r="X2" s="20"/>
+      <c r="Y2" s="20"/>
+      <c r="Z2" s="20"/>
+      <c r="AD2" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="AE2" s="11"/>
-      <c r="AF2" s="11"/>
-      <c r="AG2" s="11"/>
-      <c r="AH2" s="11"/>
-      <c r="AI2" s="11"/>
-      <c r="AJ2" s="11"/>
+      <c r="AE2" s="20"/>
+      <c r="AF2" s="20"/>
+      <c r="AG2" s="20"/>
+      <c r="AH2" s="20"/>
+      <c r="AI2" s="20"/>
+      <c r="AJ2" s="20"/>
       <c r="AK2" s="8"/>
       <c r="AL2" s="8"/>
     </row>
@@ -9388,21 +9389,21 @@
       </c>
     </row>
     <row r="48" spans="2:23" x14ac:dyDescent="0.35">
-      <c r="B48" s="10" t="s">
+      <c r="B48" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="C48" s="10"/>
-      <c r="D48" s="10"/>
-      <c r="E48" s="10"/>
+      <c r="C48" s="22"/>
+      <c r="D48" s="22"/>
+      <c r="E48" s="22"/>
     </row>
     <row r="50" spans="14:26" x14ac:dyDescent="0.35">
-      <c r="N50" s="9" t="s">
+      <c r="N50" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="O50" s="9"/>
-      <c r="P50" s="9"/>
-      <c r="Q50" s="9"/>
-      <c r="R50" s="9"/>
+      <c r="O50" s="21"/>
+      <c r="P50" s="21"/>
+      <c r="Q50" s="21"/>
+      <c r="R50" s="21"/>
       <c r="V50" t="s">
         <v>107</v>
       </c>
@@ -9449,13 +9450,13 @@
       </c>
     </row>
     <row r="58" spans="14:26" x14ac:dyDescent="0.35">
-      <c r="N58" s="9" t="s">
+      <c r="N58" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="O58" s="9"/>
-      <c r="P58" s="9"/>
-      <c r="Q58" s="9"/>
-      <c r="R58" s="9"/>
+      <c r="O58" s="21"/>
+      <c r="P58" s="21"/>
+      <c r="Q58" s="21"/>
+      <c r="R58" s="21"/>
     </row>
     <row r="60" spans="14:26" x14ac:dyDescent="0.35">
       <c r="N60" t="s">
@@ -9484,14 +9485,14 @@
       <c r="N64" t="s">
         <v>16</v>
       </c>
-      <c r="U64" s="13" t="s">
+      <c r="U64" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="V64" s="14"/>
-      <c r="W64" s="14"/>
-      <c r="X64" s="14"/>
-      <c r="Y64" s="14"/>
-      <c r="Z64" s="14"/>
+      <c r="V64" s="10"/>
+      <c r="W64" s="10"/>
+      <c r="X64" s="10"/>
+      <c r="Y64" s="10"/>
+      <c r="Z64" s="10"/>
     </row>
     <row r="65" spans="14:22" x14ac:dyDescent="0.35">
       <c r="N65" t="s">
@@ -9547,109 +9548,77 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4975E7A9-7752-4B1C-B186-BBC7B2B57660}">
-  <dimension ref="C3:K22"/>
+  <dimension ref="C3:C16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="3" spans="3:3" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="11" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="4" spans="3:3" ht="16" x14ac:dyDescent="0.35">
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="12" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="5" spans="3:3" ht="16" x14ac:dyDescent="0.35">
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="12" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="6" spans="3:3" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="11" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="7" spans="3:3" ht="16" x14ac:dyDescent="0.35">
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="12" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="8" spans="3:3" ht="16" x14ac:dyDescent="0.35">
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="13" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="9" spans="3:3" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="11" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="10" spans="3:3" ht="16" x14ac:dyDescent="0.35">
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="14" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="11" spans="3:3" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="11" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="12" spans="3:3" ht="16" x14ac:dyDescent="0.35">
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="12" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="13" spans="3:3" ht="16" x14ac:dyDescent="0.35">
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="15" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="14" spans="3:3" ht="16" x14ac:dyDescent="0.35">
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="15" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="15" spans="3:3" ht="16" x14ac:dyDescent="0.35">
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="15" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="16" spans="3:3" ht="16" x14ac:dyDescent="0.35">
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="12" t="s">
         <v>129</v>
-      </c>
-    </row>
-    <row r="19" spans="9:11" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="20" spans="9:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="I20" s="20"/>
-      <c r="J20" s="21" t="s">
-        <v>130</v>
-      </c>
-      <c r="K20" s="21" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="21" spans="9:11" ht="224.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="I21" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="J21" s="23" t="s">
-        <v>133</v>
-      </c>
-      <c r="K21" s="23" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="22" spans="9:11" ht="304.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="I22" s="22" t="s">
-        <v>135</v>
-      </c>
-      <c r="J22" s="23" t="s">
-        <v>136</v>
-      </c>
-      <c r="K22" s="23" t="s">
-        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -9658,6 +9627,52 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39DCE81F-EE57-4F7E-9711-CBC0F05A507F}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="37.81640625" customWidth="1"/>
+    <col min="2" max="2" width="43.26953125" customWidth="1"/>
+    <col min="3" max="3" width="45.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="16"/>
+      <c r="B1" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="32.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>133</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="48.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>137</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0681933B-6749-4A17-925F-E9EB49A25785}">
   <dimension ref="B2:G29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -9671,14 +9686,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
@@ -9781,14 +9796,14 @@
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="21"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
@@ -10022,26 +10037,26 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E55B153B-88FB-4A10-8D3D-E1FB39BC69A3}">
   <dimension ref="B4:E17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="4" spans="2:5" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
     </row>
     <row r="17" spans="2:5" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -10053,7 +10068,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CF64B0D-5B81-4205-8202-EA1D03B0667B}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
Create PatternCluster.sql - dbo.PattenCluster
</commit_message>
<xml_diff>
--- a/1.training_model/supplementary/1. Flowchart ML development.xlsx
+++ b/1.training_model/supplementary/1. Flowchart ML development.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{172331D7-7552-4EE9-A798-6093142F629F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{A3A45E78-3C42-44AE-93A4-41B09245FE7F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A3A45E78-3C42-44AE-93A4-41B09245FE7F}"/>
   </bookViews>
   <sheets>
     <sheet name="Flowchart ML" sheetId="1" r:id="rId1"/>
@@ -766,6 +766,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -774,9 +777,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -9338,40 +9338,40 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:38" x14ac:dyDescent="0.35">
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="N2" s="20" t="s">
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
+      <c r="N2" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="O2" s="20"/>
-      <c r="P2" s="20"/>
-      <c r="Q2" s="20"/>
-      <c r="R2" s="20"/>
-      <c r="V2" s="20" t="s">
+      <c r="O2" s="21"/>
+      <c r="P2" s="21"/>
+      <c r="Q2" s="21"/>
+      <c r="R2" s="21"/>
+      <c r="V2" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="W2" s="20"/>
-      <c r="X2" s="20"/>
-      <c r="Y2" s="20"/>
-      <c r="Z2" s="20"/>
-      <c r="AD2" s="20" t="s">
+      <c r="W2" s="21"/>
+      <c r="X2" s="21"/>
+      <c r="Y2" s="21"/>
+      <c r="Z2" s="21"/>
+      <c r="AD2" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="AE2" s="20"/>
-      <c r="AF2" s="20"/>
-      <c r="AG2" s="20"/>
-      <c r="AH2" s="20"/>
-      <c r="AI2" s="20"/>
-      <c r="AJ2" s="20"/>
+      <c r="AE2" s="21"/>
+      <c r="AF2" s="21"/>
+      <c r="AG2" s="21"/>
+      <c r="AH2" s="21"/>
+      <c r="AI2" s="21"/>
+      <c r="AJ2" s="21"/>
       <c r="AK2" s="8"/>
       <c r="AL2" s="8"/>
     </row>
@@ -9389,21 +9389,21 @@
       </c>
     </row>
     <row r="48" spans="2:23" x14ac:dyDescent="0.35">
-      <c r="B48" s="22" t="s">
+      <c r="B48" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="C48" s="22"/>
-      <c r="D48" s="22"/>
-      <c r="E48" s="22"/>
+      <c r="C48" s="23"/>
+      <c r="D48" s="23"/>
+      <c r="E48" s="23"/>
     </row>
     <row r="50" spans="14:26" x14ac:dyDescent="0.35">
-      <c r="N50" s="21" t="s">
+      <c r="N50" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="O50" s="21"/>
-      <c r="P50" s="21"/>
-      <c r="Q50" s="21"/>
-      <c r="R50" s="21"/>
+      <c r="O50" s="22"/>
+      <c r="P50" s="22"/>
+      <c r="Q50" s="22"/>
+      <c r="R50" s="22"/>
       <c r="V50" t="s">
         <v>107</v>
       </c>
@@ -9450,13 +9450,13 @@
       </c>
     </row>
     <row r="58" spans="14:26" x14ac:dyDescent="0.35">
-      <c r="N58" s="21" t="s">
+      <c r="N58" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="O58" s="21"/>
-      <c r="P58" s="21"/>
-      <c r="Q58" s="21"/>
-      <c r="R58" s="21"/>
+      <c r="O58" s="22"/>
+      <c r="P58" s="22"/>
+      <c r="Q58" s="22"/>
+      <c r="R58" s="22"/>
     </row>
     <row r="60" spans="14:26" x14ac:dyDescent="0.35">
       <c r="N60" t="s">
@@ -9686,14 +9686,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
@@ -9796,14 +9796,14 @@
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="21"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="21"/>
-      <c r="G12" s="21"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
@@ -10043,20 +10043,20 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="4" spans="2:5" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
     </row>
     <row r="17" spans="2:5" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="B17" s="23" t="s">
+      <c r="B17" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="23"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
refine slide update - finalize
</commit_message>
<xml_diff>
--- a/1.training_model/supplementary/1. Flowchart ML development.xlsx
+++ b/1.training_model/supplementary/1. Flowchart ML development.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sitisyaziyah\source\repos\DeviceCluster\1.training_model\supplementary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41250020-B058-42D0-876A-187674F05510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D626908-1957-4AE0-90C0-53A719F552F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A3A45E78-3C42-44AE-93A4-41B09245FE7F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3A45E78-3C42-44AE-93A4-41B09245FE7F}"/>
   </bookViews>
   <sheets>
     <sheet name="Flowchart ML" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="140">
   <si>
     <t>ALPHA_PREFIX_WEIGHT     = 0.65</t>
   </si>
@@ -545,7 +545,10 @@
     <t>dbo.DeviceReviewQueue</t>
   </si>
   <si>
-    <t>Current Workflow Application [28/08/2026]</t>
+    <t>ML pipeline workflow</t>
+  </si>
+  <si>
+    <t>Model Integration [28/08/2026]</t>
   </si>
 </sst>
 </file>
@@ -618,7 +621,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -652,6 +655,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -720,7 +729,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -768,16 +777,26 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -801,7 +820,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>314655</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>181085</xdr:rowOff>
@@ -882,13 +901,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>149189</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>54230</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>157522</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>180260</xdr:rowOff>
@@ -941,7 +960,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
+      <xdr:col>17</xdr:col>
       <xdr:colOff>102798</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>178274</xdr:rowOff>
@@ -1036,7 +1055,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>250265</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>177085</xdr:rowOff>
@@ -1125,7 +1144,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>449303</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>122757</xdr:rowOff>
@@ -1220,7 +1239,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>407393</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>24229</xdr:rowOff>
@@ -1301,7 +1320,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>14</xdr:col>
       <xdr:colOff>213129</xdr:colOff>
       <xdr:row>34</xdr:row>
       <xdr:rowOff>979</xdr:rowOff>
@@ -1375,13 +1394,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>149189</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>146635</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>166449</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>181449</xdr:rowOff>
@@ -1434,13 +1453,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>162862</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>46824</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>166449</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>125932</xdr:rowOff>
@@ -1493,13 +1512,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>162862</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>174479</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>166772</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>27404</xdr:rowOff>
@@ -1552,13 +1571,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>317674</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>66502</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>410568</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>9429</xdr:rowOff>
@@ -1608,7 +1627,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>14</xdr:col>
       <xdr:colOff>203326</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>6255</xdr:rowOff>
@@ -1689,7 +1708,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>19</xdr:col>
       <xdr:colOff>379604</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>17461</xdr:rowOff>
@@ -1767,13 +1786,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>19</xdr:col>
       <xdr:colOff>540161</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>66503</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
+      <xdr:col>21</xdr:col>
       <xdr:colOff>87656</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>17461</xdr:rowOff>
@@ -1823,13 +1842,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>317674</xdr:colOff>
       <xdr:row>31</xdr:row>
       <xdr:rowOff>87628</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>333827</xdr:colOff>
       <xdr:row>34</xdr:row>
       <xdr:rowOff>979</xdr:rowOff>
@@ -1882,7 +1901,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>19</xdr:col>
       <xdr:colOff>567293</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>159701</xdr:rowOff>
@@ -1956,13 +1975,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
+      <xdr:col>21</xdr:col>
       <xdr:colOff>76523</xdr:colOff>
       <xdr:row>31</xdr:row>
       <xdr:rowOff>95659</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
+      <xdr:col>21</xdr:col>
       <xdr:colOff>87656</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>162876</xdr:rowOff>
@@ -2015,13 +2034,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>333827</xdr:colOff>
       <xdr:row>35</xdr:row>
       <xdr:rowOff>68848</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
+      <xdr:col>21</xdr:col>
       <xdr:colOff>76523</xdr:colOff>
       <xdr:row>35</xdr:row>
       <xdr:rowOff>86245</xdr:rowOff>
@@ -2074,13 +2093,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>142875</xdr:colOff>
       <xdr:row>36</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>150264</xdr:colOff>
       <xdr:row>39</xdr:row>
       <xdr:rowOff>173264</xdr:rowOff>
@@ -2132,7 +2151,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
+      <xdr:col>17</xdr:col>
       <xdr:colOff>37224</xdr:colOff>
       <xdr:row>39</xdr:row>
       <xdr:rowOff>173264</xdr:rowOff>
@@ -2206,7 +2225,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
+      <xdr:col>27</xdr:col>
       <xdr:colOff>501671</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>17114</xdr:rowOff>
@@ -2275,13 +2294,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
+      <xdr:col>28</xdr:col>
       <xdr:colOff>450145</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>103080</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>28</xdr:col>
       <xdr:colOff>450597</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>68505</xdr:rowOff>
@@ -2334,7 +2353,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
+      <xdr:col>27</xdr:col>
       <xdr:colOff>23987</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>3143</xdr:rowOff>
@@ -2408,7 +2427,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
+      <xdr:col>27</xdr:col>
       <xdr:colOff>199906</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>65330</xdr:rowOff>
@@ -2485,7 +2504,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
+      <xdr:col>27</xdr:col>
       <xdr:colOff>396935</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>25727</xdr:rowOff>
@@ -2583,13 +2602,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
+      <xdr:col>28</xdr:col>
       <xdr:colOff>450474</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>164664</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>28</xdr:col>
       <xdr:colOff>454795</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>3143</xdr:rowOff>
@@ -2642,13 +2661,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
+      <xdr:col>28</xdr:col>
       <xdr:colOff>455711</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>89109</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>28</xdr:col>
       <xdr:colOff>458327</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>28902</xdr:rowOff>
@@ -2701,7 +2720,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
+      <xdr:col>27</xdr:col>
       <xdr:colOff>416072</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>107293</xdr:rowOff>
@@ -2798,13 +2817,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
+      <xdr:col>28</xdr:col>
       <xdr:colOff>470171</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>98054</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>28</xdr:col>
       <xdr:colOff>477464</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>104118</xdr:rowOff>
@@ -2857,7 +2876,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
+      <xdr:col>26</xdr:col>
       <xdr:colOff>564013</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>8913</xdr:rowOff>
@@ -2931,13 +2950,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
+      <xdr:col>28</xdr:col>
       <xdr:colOff>458327</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>108500</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>28</xdr:col>
       <xdr:colOff>470171</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>12088</xdr:rowOff>
@@ -2990,7 +3009,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
+      <xdr:col>26</xdr:col>
       <xdr:colOff>581476</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>122612</xdr:rowOff>
@@ -3064,13 +3083,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
+      <xdr:col>28</xdr:col>
       <xdr:colOff>477464</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>5123</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>28</xdr:col>
       <xdr:colOff>487634</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>125787</xdr:rowOff>
@@ -3123,16 +3142,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>590550</xdr:colOff>
       <xdr:row>75</xdr:row>
       <xdr:rowOff>149225</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
+      <xdr:col>22</xdr:col>
       <xdr:colOff>133882</xdr:colOff>
       <xdr:row>90</xdr:row>
-      <xdr:rowOff>28937</xdr:rowOff>
+      <xdr:rowOff>25762</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3172,16 +3191,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>511175</xdr:colOff>
       <xdr:row>91</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
+      <xdr:col>22</xdr:col>
       <xdr:colOff>171450</xdr:colOff>
       <xdr:row>105</xdr:row>
-      <xdr:rowOff>30037</xdr:rowOff>
+      <xdr:rowOff>26862</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3221,14 +3240,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>38100</xdr:colOff>
       <xdr:row>52</xdr:row>
       <xdr:rowOff>101600</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>102290</xdr:colOff>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>105465</xdr:colOff>
       <xdr:row>74</xdr:row>
       <xdr:rowOff>57699</xdr:rowOff>
     </xdr:to>
@@ -3270,16 +3289,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
+      <xdr:col>20</xdr:col>
       <xdr:colOff>251318</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>18804</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>390526</xdr:colOff>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>387351</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>141782</xdr:rowOff>
+      <xdr:rowOff>144957</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3320,7 +3339,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>22</xdr:col>
+      <xdr:col>35</xdr:col>
       <xdr:colOff>145772</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>19739</xdr:rowOff>
@@ -3393,7 +3412,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>22</xdr:col>
+      <xdr:col>35</xdr:col>
       <xdr:colOff>487878</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>70523</xdr:rowOff>
@@ -3467,7 +3486,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>22</xdr:col>
+      <xdr:col>35</xdr:col>
       <xdr:colOff>142994</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>8612</xdr:rowOff>
@@ -3548,7 +3567,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>22</xdr:col>
+      <xdr:col>35</xdr:col>
       <xdr:colOff>128706</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>14168</xdr:rowOff>
@@ -3629,7 +3648,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>21</xdr:col>
+      <xdr:col>34</xdr:col>
       <xdr:colOff>477006</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>3327</xdr:rowOff>
@@ -3703,7 +3722,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>21</xdr:col>
+      <xdr:col>34</xdr:col>
       <xdr:colOff>571857</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>118817</xdr:rowOff>
@@ -3777,13 +3796,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>23</xdr:col>
+      <xdr:col>36</xdr:col>
       <xdr:colOff>401877</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>105705</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
+      <xdr:col>36</xdr:col>
       <xdr:colOff>407451</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>67348</xdr:rowOff>
@@ -3836,13 +3855,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>23</xdr:col>
+      <xdr:col>36</xdr:col>
       <xdr:colOff>399099</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>153314</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
+      <xdr:col>36</xdr:col>
       <xdr:colOff>407451</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>11787</xdr:rowOff>
@@ -3895,13 +3914,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>23</xdr:col>
+      <xdr:col>36</xdr:col>
       <xdr:colOff>393187</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>92472</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
+      <xdr:col>36</xdr:col>
       <xdr:colOff>399099</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>121992</xdr:rowOff>
@@ -3954,13 +3973,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>23</xdr:col>
+      <xdr:col>36</xdr:col>
       <xdr:colOff>384811</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>29364</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
+      <xdr:col>36</xdr:col>
       <xdr:colOff>393187</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>10993</xdr:rowOff>
@@ -4013,13 +4032,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>23</xdr:col>
+      <xdr:col>36</xdr:col>
       <xdr:colOff>384811</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>91678</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
+      <xdr:col>36</xdr:col>
       <xdr:colOff>386339</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>6502</xdr:rowOff>
@@ -4072,7 +4091,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>22</xdr:col>
+      <xdr:col>35</xdr:col>
       <xdr:colOff>119976</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>177680</xdr:rowOff>
@@ -4153,7 +4172,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>21</xdr:col>
+      <xdr:col>34</xdr:col>
       <xdr:colOff>469007</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>11914</xdr:rowOff>
@@ -4227,13 +4246,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>23</xdr:col>
+      <xdr:col>36</xdr:col>
       <xdr:colOff>382431</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>92468</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
+      <xdr:col>36</xdr:col>
       <xdr:colOff>386339</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>2261</xdr:rowOff>
@@ -4286,13 +4305,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>23</xdr:col>
+      <xdr:col>36</xdr:col>
       <xdr:colOff>375165</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>82947</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
+      <xdr:col>36</xdr:col>
       <xdr:colOff>382431</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>8739</xdr:rowOff>
@@ -4345,13 +4364,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>23</xdr:col>
+      <xdr:col>36</xdr:col>
       <xdr:colOff>375165</xdr:colOff>
       <xdr:row>31</xdr:row>
       <xdr:rowOff>94706</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
+      <xdr:col>36</xdr:col>
       <xdr:colOff>383332</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>9136</xdr:rowOff>
@@ -4404,7 +4423,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>22</xdr:col>
+      <xdr:col>35</xdr:col>
       <xdr:colOff>141188</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>5961</xdr:rowOff>
@@ -4473,7 +4492,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>34</xdr:col>
+      <xdr:col>47</xdr:col>
       <xdr:colOff>61092</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>85189</xdr:rowOff>
@@ -4577,7 +4596,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>34</xdr:col>
+      <xdr:col>47</xdr:col>
       <xdr:colOff>398389</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>87801</xdr:rowOff>
@@ -4651,7 +4670,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>34</xdr:col>
+      <xdr:col>47</xdr:col>
       <xdr:colOff>53731</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>26656</xdr:rowOff>
@@ -4732,7 +4751,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>34</xdr:col>
+      <xdr:col>47</xdr:col>
       <xdr:colOff>53551</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>179139</xdr:rowOff>
@@ -4813,13 +4832,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>35</xdr:col>
+      <xdr:col>48</xdr:col>
       <xdr:colOff>318867</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>154113</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>35</xdr:col>
+      <xdr:col>48</xdr:col>
       <xdr:colOff>319632</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>87801</xdr:rowOff>
@@ -4872,13 +4891,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>35</xdr:col>
+      <xdr:col>48</xdr:col>
       <xdr:colOff>311506</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>168430</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>35</xdr:col>
+      <xdr:col>48</xdr:col>
       <xdr:colOff>319632</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>26656</xdr:rowOff>
@@ -4931,13 +4950,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>35</xdr:col>
+      <xdr:col>48</xdr:col>
       <xdr:colOff>311326</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>96667</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>35</xdr:col>
+      <xdr:col>48</xdr:col>
       <xdr:colOff>311506</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>179139</xdr:rowOff>
@@ -4991,7 +5010,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>34</xdr:col>
+      <xdr:col>47</xdr:col>
       <xdr:colOff>55112</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>176493</xdr:rowOff>
@@ -5072,13 +5091,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>35</xdr:col>
+      <xdr:col>48</xdr:col>
       <xdr:colOff>311326</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>65218</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>35</xdr:col>
+      <xdr:col>48</xdr:col>
       <xdr:colOff>312887</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>176493</xdr:rowOff>
@@ -5132,13 +5151,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>35</xdr:col>
+      <xdr:col>48</xdr:col>
       <xdr:colOff>310423</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>66678</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>35</xdr:col>
+      <xdr:col>48</xdr:col>
       <xdr:colOff>321281</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>107555</xdr:rowOff>
@@ -5192,7 +5211,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>33</xdr:col>
+      <xdr:col>46</xdr:col>
       <xdr:colOff>174334</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>107555</xdr:rowOff>
@@ -5345,7 +5364,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>30</xdr:col>
+      <xdr:col>43</xdr:col>
       <xdr:colOff>293601</xdr:colOff>
       <xdr:row>77</xdr:row>
       <xdr:rowOff>163294</xdr:rowOff>
@@ -5431,7 +5450,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>31</xdr:col>
+      <xdr:col>44</xdr:col>
       <xdr:colOff>15599</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>180813</xdr:rowOff>
@@ -5501,7 +5520,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>37</xdr:col>
+      <xdr:col>50</xdr:col>
       <xdr:colOff>344004</xdr:colOff>
       <xdr:row>31</xdr:row>
       <xdr:rowOff>47623</xdr:rowOff>
@@ -5570,13 +5589,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>32</xdr:col>
+      <xdr:col>45</xdr:col>
       <xdr:colOff>71544</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>111187</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>33</xdr:col>
+      <xdr:col>46</xdr:col>
       <xdr:colOff>174334</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>180812</xdr:rowOff>
@@ -5629,13 +5648,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>37</xdr:col>
+      <xdr:col>50</xdr:col>
       <xdr:colOff>478081</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>111188</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>38</xdr:col>
+      <xdr:col>51</xdr:col>
       <xdr:colOff>399949</xdr:colOff>
       <xdr:row>31</xdr:row>
       <xdr:rowOff>47623</xdr:rowOff>
@@ -5688,7 +5707,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>31</xdr:col>
+      <xdr:col>44</xdr:col>
       <xdr:colOff>20654</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>182744</xdr:rowOff>
@@ -5757,7 +5776,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>30</xdr:col>
+      <xdr:col>43</xdr:col>
       <xdr:colOff>449178</xdr:colOff>
       <xdr:row>36</xdr:row>
       <xdr:rowOff>150106</xdr:rowOff>
@@ -5826,13 +5845,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>32</xdr:col>
+      <xdr:col>45</xdr:col>
       <xdr:colOff>66098</xdr:colOff>
       <xdr:row>35</xdr:row>
       <xdr:rowOff>79442</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>32</xdr:col>
+      <xdr:col>45</xdr:col>
       <xdr:colOff>76599</xdr:colOff>
       <xdr:row>36</xdr:row>
       <xdr:rowOff>150106</xdr:rowOff>
@@ -5886,13 +5905,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>30</xdr:col>
+      <xdr:col>43</xdr:col>
       <xdr:colOff>184298</xdr:colOff>
       <xdr:row>37</xdr:row>
       <xdr:rowOff>95620</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
+      <xdr:col>43</xdr:col>
       <xdr:colOff>449178</xdr:colOff>
       <xdr:row>38</xdr:row>
       <xdr:rowOff>145632</xdr:rowOff>
@@ -5945,7 +5964,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>29</xdr:col>
+      <xdr:col>42</xdr:col>
       <xdr:colOff>132218</xdr:colOff>
       <xdr:row>38</xdr:row>
       <xdr:rowOff>145633</xdr:rowOff>
@@ -6014,7 +6033,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>33</xdr:col>
+      <xdr:col>46</xdr:col>
       <xdr:colOff>235603</xdr:colOff>
       <xdr:row>38</xdr:row>
       <xdr:rowOff>115488</xdr:rowOff>
@@ -6083,13 +6102,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>33</xdr:col>
+      <xdr:col>46</xdr:col>
       <xdr:colOff>280149</xdr:colOff>
       <xdr:row>37</xdr:row>
       <xdr:rowOff>95621</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>34</xdr:col>
+      <xdr:col>47</xdr:col>
       <xdr:colOff>287684</xdr:colOff>
       <xdr:row>38</xdr:row>
       <xdr:rowOff>115488</xdr:rowOff>
@@ -6142,7 +6161,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>29</xdr:col>
+      <xdr:col>42</xdr:col>
       <xdr:colOff>100492</xdr:colOff>
       <xdr:row>46</xdr:row>
       <xdr:rowOff>106344</xdr:rowOff>
@@ -6216,7 +6235,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>29</xdr:col>
+      <xdr:col>42</xdr:col>
       <xdr:colOff>102539</xdr:colOff>
       <xdr:row>50</xdr:row>
       <xdr:rowOff>73749</xdr:rowOff>
@@ -6290,13 +6309,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>30</xdr:col>
+      <xdr:col>43</xdr:col>
       <xdr:colOff>165788</xdr:colOff>
       <xdr:row>40</xdr:row>
       <xdr:rowOff>40738</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
+      <xdr:col>43</xdr:col>
       <xdr:colOff>184978</xdr:colOff>
       <xdr:row>41</xdr:row>
       <xdr:rowOff>76672</xdr:rowOff>
@@ -6350,13 +6369,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>30</xdr:col>
+      <xdr:col>43</xdr:col>
       <xdr:colOff>153556</xdr:colOff>
       <xdr:row>48</xdr:row>
       <xdr:rowOff>9956</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
+      <xdr:col>43</xdr:col>
       <xdr:colOff>158778</xdr:colOff>
       <xdr:row>50</xdr:row>
       <xdr:rowOff>76924</xdr:rowOff>
@@ -6410,7 +6429,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>33</xdr:col>
+      <xdr:col>46</xdr:col>
       <xdr:colOff>5496</xdr:colOff>
       <xdr:row>41</xdr:row>
       <xdr:rowOff>31014</xdr:rowOff>
@@ -6499,7 +6518,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>33</xdr:col>
+      <xdr:col>46</xdr:col>
       <xdr:colOff>254317</xdr:colOff>
       <xdr:row>44</xdr:row>
       <xdr:rowOff>92276</xdr:rowOff>
@@ -6568,13 +6587,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>34</xdr:col>
+      <xdr:col>47</xdr:col>
       <xdr:colOff>288363</xdr:colOff>
       <xdr:row>40</xdr:row>
       <xdr:rowOff>10593</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>34</xdr:col>
+      <xdr:col>47</xdr:col>
       <xdr:colOff>307657</xdr:colOff>
       <xdr:row>41</xdr:row>
       <xdr:rowOff>31014</xdr:rowOff>
@@ -6628,13 +6647,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>34</xdr:col>
+      <xdr:col>47</xdr:col>
       <xdr:colOff>311595</xdr:colOff>
       <xdr:row>42</xdr:row>
       <xdr:rowOff>117906</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>34</xdr:col>
+      <xdr:col>47</xdr:col>
       <xdr:colOff>317371</xdr:colOff>
       <xdr:row>44</xdr:row>
       <xdr:rowOff>92276</xdr:rowOff>
@@ -6688,13 +6707,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>32</xdr:col>
+      <xdr:col>45</xdr:col>
       <xdr:colOff>71544</xdr:colOff>
       <xdr:row>32</xdr:row>
       <xdr:rowOff>77511</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>32</xdr:col>
+      <xdr:col>45</xdr:col>
       <xdr:colOff>76599</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>182744</xdr:rowOff>
@@ -6748,7 +6767,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>37</xdr:col>
+      <xdr:col>50</xdr:col>
       <xdr:colOff>177320</xdr:colOff>
       <xdr:row>34</xdr:row>
       <xdr:rowOff>27198</xdr:rowOff>
@@ -6826,13 +6845,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>38</xdr:col>
+      <xdr:col>51</xdr:col>
       <xdr:colOff>399949</xdr:colOff>
       <xdr:row>32</xdr:row>
       <xdr:rowOff>128252</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>38</xdr:col>
+      <xdr:col>51</xdr:col>
       <xdr:colOff>400576</xdr:colOff>
       <xdr:row>34</xdr:row>
       <xdr:rowOff>27198</xdr:rowOff>
@@ -6886,7 +6905,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>33</xdr:col>
+      <xdr:col>46</xdr:col>
       <xdr:colOff>250001</xdr:colOff>
       <xdr:row>47</xdr:row>
       <xdr:rowOff>169216</xdr:rowOff>
@@ -6956,13 +6975,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>34</xdr:col>
+      <xdr:col>47</xdr:col>
       <xdr:colOff>304094</xdr:colOff>
       <xdr:row>45</xdr:row>
       <xdr:rowOff>170334</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>34</xdr:col>
+      <xdr:col>47</xdr:col>
       <xdr:colOff>308410</xdr:colOff>
       <xdr:row>47</xdr:row>
       <xdr:rowOff>169216</xdr:rowOff>
@@ -7016,7 +7035,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>23</xdr:col>
+      <xdr:col>36</xdr:col>
       <xdr:colOff>597514</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>160697</xdr:rowOff>
@@ -7076,7 +7095,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>28</xdr:col>
+      <xdr:col>41</xdr:col>
       <xdr:colOff>286182</xdr:colOff>
       <xdr:row>41</xdr:row>
       <xdr:rowOff>76672</xdr:rowOff>
@@ -7212,13 +7231,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>30</xdr:col>
+      <xdr:col>43</xdr:col>
       <xdr:colOff>153556</xdr:colOff>
       <xdr:row>44</xdr:row>
       <xdr:rowOff>143704</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
+      <xdr:col>43</xdr:col>
       <xdr:colOff>166396</xdr:colOff>
       <xdr:row>46</xdr:row>
       <xdr:rowOff>106344</xdr:rowOff>
@@ -7272,7 +7291,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>28</xdr:col>
+      <xdr:col>41</xdr:col>
       <xdr:colOff>303716</xdr:colOff>
       <xdr:row>53</xdr:row>
       <xdr:rowOff>120484</xdr:rowOff>
@@ -7420,13 +7439,13 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>30</xdr:col>
+      <xdr:col>43</xdr:col>
       <xdr:colOff>151938</xdr:colOff>
       <xdr:row>51</xdr:row>
       <xdr:rowOff>165264</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
+      <xdr:col>43</xdr:col>
       <xdr:colOff>158778</xdr:colOff>
       <xdr:row>53</xdr:row>
       <xdr:rowOff>120484</xdr:rowOff>
@@ -7480,13 +7499,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>32</xdr:col>
+      <xdr:col>45</xdr:col>
       <xdr:colOff>381000</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>138546</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>38</xdr:col>
+      <xdr:col>51</xdr:col>
       <xdr:colOff>346363</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>34636</xdr:rowOff>
@@ -7546,7 +7565,7 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>32</xdr:col>
+      <xdr:col>45</xdr:col>
       <xdr:colOff>88347</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>176695</xdr:rowOff>
@@ -7613,6 +7632,56 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>565934</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>46475</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>245260</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>129874</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="24" name="Picture 23">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{70776F89-5186-42C3-88EC-C7EF0E527762}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1172070" y="912384"/>
+          <a:ext cx="5134554" cy="7703399"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -9486,226 +9555,249 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38AA77DD-8AB1-42B3-B673-04FA8231C115}">
-  <dimension ref="B2:AP84"/>
+  <dimension ref="B2:BF84"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="12" max="12" width="2.1796875" style="2" customWidth="1"/>
-    <col min="20" max="20" width="2.6328125" style="2" customWidth="1"/>
-    <col min="27" max="27" width="8.7265625" customWidth="1"/>
-    <col min="28" max="28" width="2.6328125" style="2" customWidth="1"/>
+    <col min="12" max="12" width="8.7265625" customWidth="1"/>
+    <col min="13" max="13" width="1.7265625" style="2" customWidth="1"/>
+    <col min="25" max="25" width="2.1796875" style="2" customWidth="1"/>
+    <col min="33" max="33" width="2.6328125" style="2" customWidth="1"/>
+    <col min="40" max="40" width="8.7265625" customWidth="1"/>
+    <col min="41" max="41" width="2.6328125" style="2" customWidth="1"/>
+    <col min="57" max="57" width="4.453125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:42" x14ac:dyDescent="0.35">
-      <c r="B2" s="21" t="s">
+    <row r="2" spans="2:58" x14ac:dyDescent="0.35">
+      <c r="B2" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="26"/>
+      <c r="O2" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
-      <c r="N2" s="21" t="s">
+      <c r="P2" s="19"/>
+      <c r="Q2" s="19"/>
+      <c r="R2" s="19"/>
+      <c r="S2" s="19"/>
+      <c r="T2" s="19"/>
+      <c r="U2" s="19"/>
+      <c r="V2" s="19"/>
+      <c r="W2" s="19"/>
+      <c r="AA2" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="O2" s="21"/>
-      <c r="P2" s="21"/>
-      <c r="Q2" s="21"/>
-      <c r="R2" s="21"/>
-      <c r="V2" s="21" t="s">
+      <c r="AB2" s="19"/>
+      <c r="AC2" s="19"/>
+      <c r="AD2" s="19"/>
+      <c r="AE2" s="19"/>
+      <c r="AI2" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="W2" s="21"/>
-      <c r="X2" s="21"/>
-      <c r="Y2" s="21"/>
-      <c r="Z2" s="21"/>
-      <c r="AD2" s="21" t="s">
-        <v>138</v>
-      </c>
-      <c r="AE2" s="21"/>
-      <c r="AF2" s="21"/>
-      <c r="AG2" s="21"/>
-      <c r="AH2" s="21"/>
-      <c r="AI2" s="21"/>
-      <c r="AJ2" s="21"/>
-      <c r="AK2" s="21"/>
-      <c r="AL2" s="21"/>
-      <c r="AM2" s="21"/>
-      <c r="AN2" s="21"/>
-      <c r="AO2" s="21"/>
-      <c r="AP2" s="21"/>
+      <c r="AJ2" s="19"/>
+      <c r="AK2" s="19"/>
+      <c r="AL2" s="19"/>
+      <c r="AM2" s="19"/>
+      <c r="AQ2" s="19" t="s">
+        <v>139</v>
+      </c>
+      <c r="AR2" s="19"/>
+      <c r="AS2" s="19"/>
+      <c r="AT2" s="19"/>
+      <c r="AU2" s="19"/>
+      <c r="AV2" s="19"/>
+      <c r="AW2" s="19"/>
+      <c r="AX2" s="19"/>
+      <c r="AY2" s="19"/>
+      <c r="AZ2" s="19"/>
+      <c r="BA2" s="19"/>
+      <c r="BB2" s="19"/>
+      <c r="BC2" s="19"/>
+      <c r="BD2" s="24"/>
+      <c r="BE2" s="25"/>
+      <c r="BF2" s="24"/>
     </row>
-    <row r="15" spans="2:42" x14ac:dyDescent="0.35">
-      <c r="G15" s="1"/>
+    <row r="3" spans="2:58" x14ac:dyDescent="0.35">
+      <c r="BC3" s="23"/>
     </row>
-    <row r="43" spans="2:23" x14ac:dyDescent="0.35">
-      <c r="W43" t="s">
+    <row r="15" spans="2:58" x14ac:dyDescent="0.35">
+      <c r="T15" s="1"/>
+    </row>
+    <row r="43" spans="15:36" x14ac:dyDescent="0.35">
+      <c r="AJ43" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="44" spans="2:23" x14ac:dyDescent="0.35">
-      <c r="W44" t="s">
+    <row r="44" spans="15:36" x14ac:dyDescent="0.35">
+      <c r="AJ44" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="48" spans="2:23" x14ac:dyDescent="0.35">
-      <c r="B48" s="20" t="s">
+    <row r="48" spans="15:36" x14ac:dyDescent="0.35">
+      <c r="O48" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="C48" s="20"/>
-      <c r="D48" s="20"/>
-      <c r="E48" s="20"/>
+      <c r="P48" s="21"/>
+      <c r="Q48" s="21"/>
+      <c r="R48" s="21"/>
     </row>
-    <row r="50" spans="14:26" x14ac:dyDescent="0.35">
-      <c r="N50" s="19" t="s">
+    <row r="50" spans="27:39" x14ac:dyDescent="0.35">
+      <c r="AA50" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="O50" s="19"/>
-      <c r="P50" s="19"/>
-      <c r="Q50" s="19"/>
-      <c r="R50" s="19"/>
-      <c r="V50" t="s">
+      <c r="AB50" s="20"/>
+      <c r="AC50" s="20"/>
+      <c r="AD50" s="20"/>
+      <c r="AE50" s="20"/>
+      <c r="AI50" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="51" spans="14:26" x14ac:dyDescent="0.35">
-      <c r="V51" t="s">
+    <row r="51" spans="27:39" x14ac:dyDescent="0.35">
+      <c r="AI51" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="52" spans="14:26" x14ac:dyDescent="0.35">
-      <c r="N52" t="s">
+    <row r="52" spans="27:39" x14ac:dyDescent="0.35">
+      <c r="AA52" t="s">
         <v>0</v>
       </c>
-      <c r="V52" t="s">
+      <c r="AI52" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="53" spans="14:26" x14ac:dyDescent="0.35">
-      <c r="N53" t="s">
+    <row r="53" spans="27:39" x14ac:dyDescent="0.35">
+      <c r="AA53" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="14:26" x14ac:dyDescent="0.35">
-      <c r="N54" t="s">
+    <row r="54" spans="27:39" x14ac:dyDescent="0.35">
+      <c r="AA54" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="55" spans="14:26" x14ac:dyDescent="0.35">
-      <c r="N55" t="s">
+    <row r="55" spans="27:39" x14ac:dyDescent="0.35">
+      <c r="AA55" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="56" spans="14:26" x14ac:dyDescent="0.35">
-      <c r="N56" t="s">
+    <row r="56" spans="27:39" x14ac:dyDescent="0.35">
+      <c r="AA56" t="s">
         <v>4</v>
       </c>
-      <c r="V56" t="s">
+      <c r="AI56" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="57" spans="14:26" x14ac:dyDescent="0.35">
-      <c r="V57" t="s">
+    <row r="57" spans="27:39" x14ac:dyDescent="0.35">
+      <c r="AI57" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="58" spans="14:26" x14ac:dyDescent="0.35">
-      <c r="N58" s="19" t="s">
+    <row r="58" spans="27:39" x14ac:dyDescent="0.35">
+      <c r="AA58" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="O58" s="19"/>
-      <c r="P58" s="19"/>
-      <c r="Q58" s="19"/>
-      <c r="R58" s="19"/>
+      <c r="AB58" s="20"/>
+      <c r="AC58" s="20"/>
+      <c r="AD58" s="20"/>
+      <c r="AE58" s="20"/>
     </row>
-    <row r="60" spans="14:26" x14ac:dyDescent="0.35">
-      <c r="N60" t="s">
+    <row r="60" spans="27:39" x14ac:dyDescent="0.35">
+      <c r="AA60" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="61" spans="14:26" x14ac:dyDescent="0.35">
-      <c r="N61" t="s">
+    <row r="61" spans="27:39" x14ac:dyDescent="0.35">
+      <c r="AA61" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="62" spans="14:26" x14ac:dyDescent="0.35">
-      <c r="N62" t="s">
+    <row r="62" spans="27:39" x14ac:dyDescent="0.35">
+      <c r="AA62" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="63" spans="14:26" x14ac:dyDescent="0.35">
-      <c r="N63" t="s">
+    <row r="63" spans="27:39" x14ac:dyDescent="0.35">
+      <c r="AA63" t="s">
         <v>15</v>
       </c>
-      <c r="V63" t="s">
+      <c r="AI63" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="64" spans="14:26" x14ac:dyDescent="0.35">
-      <c r="N64" t="s">
+    <row r="64" spans="27:39" x14ac:dyDescent="0.35">
+      <c r="AA64" t="s">
         <v>16</v>
       </c>
-      <c r="U64" s="8" t="s">
+      <c r="AH64" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="V64" s="9"/>
-      <c r="W64" s="9"/>
-      <c r="X64" s="9"/>
-      <c r="Y64" s="9"/>
-      <c r="Z64" s="9"/>
+      <c r="AI64" s="9"/>
+      <c r="AJ64" s="9"/>
+      <c r="AK64" s="9"/>
+      <c r="AL64" s="9"/>
+      <c r="AM64" s="9"/>
     </row>
-    <row r="65" spans="14:22" x14ac:dyDescent="0.35">
-      <c r="N65" t="s">
+    <row r="65" spans="27:35" x14ac:dyDescent="0.35">
+      <c r="AA65" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="66" spans="14:22" x14ac:dyDescent="0.35">
-      <c r="N66" t="s">
+    <row r="66" spans="27:35" x14ac:dyDescent="0.35">
+      <c r="AA66" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="67" spans="14:22" x14ac:dyDescent="0.35">
-      <c r="N67" t="s">
+    <row r="67" spans="27:35" x14ac:dyDescent="0.35">
+      <c r="AA67" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="68" spans="14:22" x14ac:dyDescent="0.35">
-      <c r="N68" t="s">
+    <row r="68" spans="27:35" x14ac:dyDescent="0.35">
+      <c r="AA68" t="s">
         <v>20</v>
       </c>
-      <c r="V68" s="1" t="s">
+      <c r="AI68" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="69" spans="14:22" x14ac:dyDescent="0.35">
-      <c r="N69" t="s">
+    <row r="69" spans="27:35" x14ac:dyDescent="0.35">
+      <c r="AA69" t="s">
         <v>21</v>
       </c>
-      <c r="V69" t="s">
+      <c r="AI69" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="70" spans="14:22" x14ac:dyDescent="0.35">
-      <c r="N70" t="s">
+    <row r="70" spans="27:35" x14ac:dyDescent="0.35">
+      <c r="AA70" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="84" spans="33:33" x14ac:dyDescent="0.35">
-      <c r="AG84" t="s">
+    <row r="84" spans="46:46" x14ac:dyDescent="0.35">
+      <c r="AT84" t="s">
         <v>137</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="AD2:AP2"/>
-    <mergeCell ref="N58:R58"/>
-    <mergeCell ref="B48:E48"/>
-    <mergeCell ref="B2:J2"/>
-    <mergeCell ref="N2:R2"/>
-    <mergeCell ref="V2:Z2"/>
-    <mergeCell ref="N50:R50"/>
+  <mergeCells count="8">
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="AQ2:BC2"/>
+    <mergeCell ref="AA58:AE58"/>
+    <mergeCell ref="O48:R48"/>
+    <mergeCell ref="O2:W2"/>
+    <mergeCell ref="AA2:AE2"/>
+    <mergeCell ref="AI2:AM2"/>
+    <mergeCell ref="AA50:AE50"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -9853,14 +9945,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
@@ -9963,14 +10055,14 @@
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="19"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B14" t="s">

</xml_diff>